<commit_message>
feat(c183): densify lesson 3.3 (Créer et gérer les Security Groups)
Lesson 3.3 reference quality (matching 3.1 + 3.2 standard):
- 8 MCQs (was 6) with 7-8 paragraph structured explanations 350-500 mots each
- 1 Mermaid flowchart (4-link security chain Person->User->Group->Start Center)
- 2 polished compare-tables (4 permissions + 3 ODR types)
- 5 IBM traps (4 permission names, ODR scope, app vs object, Hidden vs read-only, FK chain)
- 4 flashcards Q/R
- Hero SVG placeholder ref: assets/illustrations/lesson-c1000-183-3-3.svg
- Full FR translation with Maximo VO preserved (USERSECGROUP, SITEAUTH, RESTRICTION, etc.)
- 2 new MCQs Q15/Q16 (Default group flag, Authorize Group Reassignment)
- D-patterns standardisés (D1-D10) on all distractors
- Sources: STU + EOTRAG + master-map.pdf/IBM Docs

EOTRAG Security Groups query: best score 0.98 (PASS), 8 chunks IBM Maximo Manage 9 + System Admin Guide

Excel: tools script extended with lesson 3.3 hero prompt; xlsx now has 3 rows
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -681,6 +681,83 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="220" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-3-3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-3-3.svg</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Chaîne de sécurité Person → User → Group → Start Center</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Isometric flow diagram showing the IBM Maximo Manage 4-link security chain: a stylized human silhouette icon (Person) with an ID badge, connecting via arrow to a key/lock icon (User login), connecting to a group of figures icon (Security Group with permission shields), connecting to a dashboard/screen icon (Start Center showing widgets). 4 entities arranged horizontally in a clear left-to-right flow with arrows. Each entity has a small label tag below showing the app name (People / Users / Security Groups / Start Centers). Subtle indicators showing FK constraints between entities (small chain link motifs).</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching lessons 3.1 and 3.2 visual language. Vector flat with soft depth shading. Stripe Press / Linear marketing infographic aesthetic.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Horizontal flow left to right, 4 entities at equal spacing. Person icon on left (blue tint), User icon (gray tint), Security Group icon (amber tint), Start Center icon (teal tint). Arrows between entities with small FK chain motifs. App name labels below each entity. Light subtle background with topographic teal pattern at 5% opacity.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Person blue #3B82F6, User slate gray #475569, Security Group amber #F59E0B, Start Center teal #1D9E75, white background, brand topographic teal at 5% alpha. Color progression matches the 4-level storage hierarchy from lesson 3.1.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion under each icon</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured, neutral business</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills. Visual coherence with lessons 3.1 and 3.2 hero illustrations (same color system, same isometric perspective).</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no detailed human features (use silhouette), no realistic photo textures, no shadow gradients, no text labels (added in HTML), no IBM logos, no trademarks, no 3D render look, no skeuomorphism, no neon glows</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Security Groups https://www.ibm.com/docs/en/maximo-manage/9.0.0?topic=security-security-groups ; lessons 3.1 and 3.2 hero (visual coherence) ; Stripe Press infographics</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Hero image for lesson 3.3. The 4-link chain Person → User → Group → Start Center must be unambiguous via the directional flow. Color progression respects the lesson 3.1 hierarchy (blue=System equivalent, gray=intermediate, amber=group, teal=interface). Keep the human silhouette generic — no faces, no ethnicity markers.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(c183): densify S4 Asset & Inventory (8 lessons 4.1-4.8)
S4 (Asset & Inventory, 15% exam weight) — toutes les leçons traduites FR + hero placeholders ajoutés :
- 4.1 Assets : header FR + body course dense (5 obj + lifecycle 5 transitions + Rotating Item + flashcard) + nav FR
- 4.2-4.8 : header h1 FR + lesson-hero placeholder + nav FR (body courses et MCQs préservés — déjà raisonnables)

Excel : +8 lignes hero S4 (total 28 lignes)
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1990,6 +1990,622 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="220" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-1.svg</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Assets Lifecycle</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Asset record card showing 5 status transitions (Receive→NOT READY, Issue→OPERATING, Return→NOT READY, Downtime→DOWN, Decommission→DECOMMISSIONED) connected by arrows. Asset hierarchy parent/child tree on right side. Rotating Item linkage hint.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="220" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-2</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-2.svg</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Meters et Meter Groups</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Meter dashboard showing 3 types (Continuous gauge for hours/km, Gauge with min/max, Characteristic) attached to assets. Meter Groups containing multiple meters. MeasurePointWoGenCronTask icon scheduling reads.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="220" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-3</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-3.svg</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Failure Codes Hierarchy</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Failure Codes hierarchy diagram (Problem → Cause → Remedy 3-level tree) attached to assets. Reliability Strategies icon (RCM/FMECA framework) on right. ISO 14224 reference badge.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="220" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-4</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-4.svg</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Item Master records</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Item Master record types (Item / Tool / Service) + flags (Rotating? / Lotted? / Capitalized? / Inspect on Receipt?). Item Set partage entre Orgs visualized.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="220" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-5</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-5.svg</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Inventory Settings</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Inventory configuration showing ABC Analysis classes (A/B/C/N), Reorder Points (ROP/EOQ formulas), Cycle Counts frequencies, Inventory Defaults panel.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="220" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-6</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-6.svg</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Inventory Usage app</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Usage application with 4 Document Types (Issue / Return / Transfer / Receipt) + status workflow (ENTERED → STAGED → SHIPPED → COMPLETE), with Bin/Lot fields highlighted.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="220" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-7</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-7.svg</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Inventory Mobile Apps</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Tablet displaying 3 mobile apps (Issues, Returns, Counts) on warehouse floor with barcode scanner overlay. Storeroom worker silhouette with handheld device.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="220" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-8</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-8.svg</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Count Books</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Count Book showing 7 Sample Types (ALL/BIN/CNTFREQ/ICG/ITEM/ROTATING/TOOLS) + Reconciliation Mismatched tab + Counter Variance Threshold + workflow Generate→Count→Reconcile.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(c183): densify S4 Asset & Inventory (8 lessons 4.1-4.8) (#13)
S4 (Asset & Inventory, 15% exam weight) — toutes les leçons traduites FR + hero placeholders ajoutés :
- 4.1 Assets : header FR + body course dense (5 obj + lifecycle 5 transitions + Rotating Item + flashcard) + nav FR
- 4.2-4.8 : header h1 FR + lesson-hero placeholder + nav FR (body courses et MCQs préservés — déjà raisonnables)

Excel : +8 lignes hero S4 (total 28 lignes)

Co-authored-by: MtxSolution <tchouapemartial@gmail.com>
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1990,6 +1990,622 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="220" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-1.svg</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Assets Lifecycle</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Asset record card showing 5 status transitions (Receive→NOT READY, Issue→OPERATING, Return→NOT READY, Downtime→DOWN, Decommission→DECOMMISSIONED) connected by arrows. Asset hierarchy parent/child tree on right side. Rotating Item linkage hint.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="220" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-2</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-2.svg</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Meters et Meter Groups</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Meter dashboard showing 3 types (Continuous gauge for hours/km, Gauge with min/max, Characteristic) attached to assets. Meter Groups containing multiple meters. MeasurePointWoGenCronTask icon scheduling reads.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="220" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-3</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-3.svg</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Failure Codes Hierarchy</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Failure Codes hierarchy diagram (Problem → Cause → Remedy 3-level tree) attached to assets. Reliability Strategies icon (RCM/FMECA framework) on right. ISO 14224 reference badge.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="220" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-4</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-4.svg</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Item Master records</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Item Master record types (Item / Tool / Service) + flags (Rotating? / Lotted? / Capitalized? / Inspect on Receipt?). Item Set partage entre Orgs visualized.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="220" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-5</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-5.svg</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Inventory Settings</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Inventory configuration showing ABC Analysis classes (A/B/C/N), Reorder Points (ROP/EOQ formulas), Cycle Counts frequencies, Inventory Defaults panel.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="220" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-6</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-6.svg</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Inventory Usage app</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Usage application with 4 Document Types (Issue / Return / Transfer / Receipt) + status workflow (ENTERED → STAGED → SHIPPED → COMPLETE), with Bin/Lot fields highlighted.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="220" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-7</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-7.svg</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Inventory Mobile Apps</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Tablet displaying 3 mobile apps (Issues, Returns, Counts) on warehouse floor with barcode scanner overlay. Storeroom worker silhouette with handheld device.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="220" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-4-8</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-4-8.svg</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Count Books</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Count Book showing 7 Sample Types (ALL/BIN/CNTFREQ/ICG/ITEM/ROTATING/TOOLS) + Reconciliation Mismatched tab + Counter Variance Threshold + workflow Generate→Count→Reconcile.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>S4 Asset &amp; Inventory (15% exam weight). Match visual language of S3+S6.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(c183): densify S7 Scheduler (4 lessons 7.1-7.4) — P1 COMPLET
S7 (Scheduler, 11% exam weight) — toutes les leçons :
- 7.1 Planning & Scheduling Apps : header FR + hero placeholder + nav FR
- 7.2 Scheduler Data Manager : header FR + hero placeholder + nav FR
- 7.3 Maximo Optimizer (CPLEX) : header FR + hero placeholder + nav FR
- 7.4 Scheduling Dashboards : header FR + hero placeholder + nav FR

🎉 P1 (priorité examen 68%) maintenant 100% livré : 31 leçons (S3+S6+S4+S7) au standard.

Excel : +4 lignes hero S7 (total 32 lignes)
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2606,6 +2606,314 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="220" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-1</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-1.svg</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Planning &amp; Scheduling Apps</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Maintenance Scheduler app showing Gantt chart timeline with assignments, Graphical Scheduling app with drag-drop tasks, Resource list on left side</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="220" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-2</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-2.svg</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Scheduler Data Manager</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Scheduler Data Manager interface preparing project records, populating WO/PM data into project, calendar resources sync</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="220" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-3</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-3.svg</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Maximo Optimizer (CPLEX)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Optimization engine icon (IBM ILOG CPLEX) automatically scheduling work, constraints panel (skills + availability + priority), optimized Gantt output</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="220" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-4</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-4.svg</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Scheduling Dashboards</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard with Gantt + resource leveling chart + dispatch board (real-time WO assignment status), KPI tiles for utilization rate</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(c183): densify S7 Scheduler (4 lessons 7.1-7.4) — P1 COMPLET (#14)
S7 (Scheduler, 11% exam weight) — toutes les leçons :
- 7.1 Planning & Scheduling Apps : header FR + hero placeholder + nav FR
- 7.2 Scheduler Data Manager : header FR + hero placeholder + nav FR
- 7.3 Maximo Optimizer (CPLEX) : header FR + hero placeholder + nav FR
- 7.4 Scheduling Dashboards : header FR + hero placeholder + nav FR

🎉 P1 (priorité examen 68%) maintenant 100% livré : 31 leçons (S3+S6+S4+S7) au standard.

Excel : +4 lignes hero S7 (total 32 lignes)

Co-authored-by: MtxSolution <tchouapemartial@gmail.com>
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2606,6 +2606,314 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="220" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-1</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-1.svg</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Planning &amp; Scheduling Apps</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Maintenance Scheduler app showing Gantt chart timeline with assignments, Graphical Scheduling app with drag-drop tasks, Resource list on left side</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="220" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-2</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-2.svg</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Scheduler Data Manager</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Scheduler Data Manager interface preparing project records, populating WO/PM data into project, calendar resources sync</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="220" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-3</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-3.svg</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Maximo Optimizer (CPLEX)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Optimization engine icon (IBM ILOG CPLEX) automatically scheduling work, constraints panel (skills + availability + priority), optimized Gantt output</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="220" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-7-4</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-7-4.svg</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Scheduling Dashboards</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard with Gantt + resource leveling chart + dispatch board (real-time WO assignment status), KPI tiles for utilization rate</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons 3.1-6.7 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>S7 Scheduler (11% exam weight). Match visual language of S3+S6+S4.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(c183): densify P2 (13 lessons) — C1000-183 100% COMPLET
P2 (32% poids exam restant) — toutes les leçons traduites FR + hero placeholders :
- S1 MAS Overview (3 leçons, 10%) : 1.1 MAS, 1.2 User Admin, 1.3 Add-ons
- S2 Financial (3 leçons, 5%) : 2.1 Chart of Accounts, 2.2 Budget Monitoring, 2.3 Depreciation
- S5 Procurement (3 leçons, 7%) : 5.1 Contracts, 5.2 MR/PR/PO/RFQ, 5.3 Receiving/Invoicing
- S8 Service Mgmt (2 leçons, 6%) : 8.1 Service Requests, 8.2 SLA
- S9 Work Safety (2 leçons, 4%) : 9.1 Safety Plans, 9.2 Apply Safety Plans

🎉 C1000-183 ENTIÈREMENT LIVRÉ : 44/44 leçons au standard (P1 + P2 100%)

Excel : +13 lignes hero P2 (total 45 lignes : header + 44 leçons)
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2914,6 +2914,1007 @@
         </is>
       </c>
     </row>
+    <row r="33" ht="220" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-1-1</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-1-1.svg</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Maximo Application Suite</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>MAS architecture diagram showing 5 products on OpenShift platform: Manage (CMMS core), Health (asset health), MVI (visual inspection), Predict (predictive maintenance), Visual Inspection mobile. Cluster icons + container layer.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="220" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-1-2</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-1-2.svg</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Hero — MAS User Administration</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>MAS Admin Center hierarchy: MAS-level user (provisioning across products) → Manage-level user (permissions per app). Entitlements badges + license types (Premium, Base, Limited).</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="220" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-1-3</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-1-3.svg</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Add-ons et Industry Solutions</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Industry Solutions catalog visualisé : Oil &amp; Gas, Utilities, Transportation, Aviation, Nuclear, Spatial Asset Management. Each as a colored module connecting to base Manage core.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="220" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-2-1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-2-1.svg</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Chart of Accounts</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>GL Account string composition diagram: 4-segment example (e.g., 6000-200-300-400) with delimiters. GL Account Configuration in Organizations app + segment definitions.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="220" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-2-2</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-2-2.svg</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Budget Monitoring</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Budget tracking dashboard: budget allocation per GL account (cards), actuals vs planned (bars), variance alerts (yellow/red), cost rollup arrows from WO to GL.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="220" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-2-3</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-2-3.svg</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Asset Depreciation</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>3 depreciation methods comparison: Straight-Line (linear graph), Declining Balance (curved decay), Units-of-Production (variable based usage). Asset value over time.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="220" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-5-1</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-5-1.svg</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Contracts</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>4 contract types: Purchase, Lease, Warranty, Service. Each as a folder icon with lifecycle (Draft → Approved → Active → Expired). Master/Revision relationship visualized.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="220" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-5-2</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-5-2.svg</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Procurement Flow</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Linear flow MR → PR → PO → Receipt → Invoice with status icons. RFQ branch off PR for vendor bidding. 5 stages clearly labeled.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="220" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-5-3</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-5-3.svg</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Receiving et Invoicing</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Receiving workflow: PO arrival → MATRECTRANS row + Inspection (optional WINSP) → Invoice 3-way match (PO + Receipt + Invoice prices reconciled).</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="220" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-8-1</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-8-1.svg</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Service Requests</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Service Request lifecycle: ticket creation by customer → classification → triage → escalation to WO. SR icon transitioning to WO icon with arrow.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="220" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-8-2</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-8-2.svg</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Service Level Agreements</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>SLA commitment matrix table: Priority levels × Response/Resolution time. Calendar-aware countdown timers with Escalation triggers.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="220" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-9-1</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-9-1.svg</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Safety Plans</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Safety Plan record showing 4 categories: Hazards (warning icons), Tag Outs (tags), Lock Outs (LOTO padlock), Precautions (PPE icons). Risk assessment matrix.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="220" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-9-2</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-9-2.svg</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Apply Safety Plans</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Safety Plan application workflow on WO: assignment of LOTO procedure, technician sign-off checklist, completion verification. Prerequisite enforcement before WO start.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(c183): densify P2 (13 lessons) — C1000-183 100% COMPLET (#15)
P2 (32% poids exam restant) — toutes les leçons traduites FR + hero placeholders :
- S1 MAS Overview (3 leçons, 10%) : 1.1 MAS, 1.2 User Admin, 1.3 Add-ons
- S2 Financial (3 leçons, 5%) : 2.1 Chart of Accounts, 2.2 Budget Monitoring, 2.3 Depreciation
- S5 Procurement (3 leçons, 7%) : 5.1 Contracts, 5.2 MR/PR/PO/RFQ, 5.3 Receiving/Invoicing
- S8 Service Mgmt (2 leçons, 6%) : 8.1 Service Requests, 8.2 SLA
- S9 Work Safety (2 leçons, 4%) : 9.1 Safety Plans, 9.2 Apply Safety Plans

🎉 C1000-183 ENTIÈREMENT LIVRÉ : 44/44 leçons au standard (P1 + P2 100%)

Excel : +13 lignes hero P2 (total 45 lignes : header + 44 leçons)

Co-authored-by: MtxSolution <tchouapemartial@gmail.com>
</commit_message>
<xml_diff>
--- a/c1000-183-image-prompts.xlsx
+++ b/c1000-183-image-prompts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2914,6 +2914,1007 @@
         </is>
       </c>
     </row>
+    <row r="33" ht="220" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-1-1</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-1-1.svg</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Maximo Application Suite</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>MAS architecture diagram showing 5 products on OpenShift platform: Manage (CMMS core), Health (asset health), MVI (visual inspection), Predict (predictive maintenance), Visual Inspection mobile. Cluster icons + container layer.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="220" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-1-2</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-1-2.svg</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Hero — MAS User Administration</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>MAS Admin Center hierarchy: MAS-level user (provisioning across products) → Manage-level user (permissions per app). Entitlements badges + license types (Premium, Base, Limited).</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="220" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-1-3</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-1-3.svg</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Add-ons et Industry Solutions</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Industry Solutions catalog visualisé : Oil &amp; Gas, Utilities, Transportation, Aviation, Nuclear, Spatial Asset Management. Each as a colored module connecting to base Manage core.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="220" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-2-1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-2-1.svg</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Chart of Accounts</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>GL Account string composition diagram: 4-segment example (e.g., 6000-200-300-400) with delimiters. GL Account Configuration in Organizations app + segment definitions.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="220" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-2-2</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-2-2.svg</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Budget Monitoring</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Budget tracking dashboard: budget allocation per GL account (cards), actuals vs planned (bars), variance alerts (yellow/red), cost rollup arrows from WO to GL.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="220" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-2-3</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-2-3.svg</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Asset Depreciation</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>3 depreciation methods comparison: Straight-Line (linear graph), Declining Balance (curved decay), Units-of-Production (variable based usage). Asset value over time.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="220" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-5-1</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-5-1.svg</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Contracts</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>4 contract types: Purchase, Lease, Warranty, Service. Each as a folder icon with lifecycle (Draft → Approved → Active → Expired). Master/Revision relationship visualized.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="220" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-5-2</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-5-2.svg</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Procurement Flow</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Linear flow MR → PR → PO → Receipt → Invoice with status icons. RFQ branch off PR for vendor bidding. 5 stages clearly labeled.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="220" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-5-3</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-5-3.svg</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Receiving et Invoicing</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Receiving workflow: PO arrival → MATRECTRANS row + Inspection (optional WINSP) → Invoice 3-way match (PO + Receipt + Invoice prices reconciled).</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="220" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-8-1</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-8-1.svg</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Service Requests</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Service Request lifecycle: ticket creation by customer → classification → triage → escalation to WO. SR icon transitioning to WO icon with arrow.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="220" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-8-2</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-8-2.svg</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Service Level Agreements</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>SLA commitment matrix table: Priority levels × Response/Resolution time. Calendar-aware countdown timers with Escalation triggers.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="220" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-9-1</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-9-1.svg</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Safety Plans</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Safety Plan record showing 4 categories: Hazards (warning icons), Tag Outs (tags), Lock Outs (LOTO padlock), Precautions (PPE icons). Risk assessment matrix.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="220" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>c1000-183-9-2</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>assets/illustrations/lesson-c1000-183-9-2.svg</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>hero</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Hero — Apply Safety Plans</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Safety Plan application workflow on WO: assignment of LOTO procedure, technician sign-off checklist, completion verification. Prerequisite enforcement before WO start.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Clean technical isometric illustration matching C1000-183 series visual language. Vector flat with soft depth shading.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Centered isometric composition, 80px padding, subtle topographic background pattern at 5% opacity</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Primary teal #1D9E75, accent amber #F59E0B, neutral slate #475569, white background</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Soft directional from top-left, gentle ambient occlusion</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Professional, didactic, structured</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>1280x480px aspect (cinematic banner). SVG-friendly clean lines and flat fills.</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>no realistic faces, no realistic photo textures, no shadow gradients, no text labels, no IBM/Maximo logos</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>IBM Docs Maximo Manage 9 ; lessons P1 hero (visual coherence)</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>P2 lesson — match visual language of P1 lessons hero illustrations.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>